<commit_message>
feat: add selenium helpers and UI modules while importing new test data and plans
</commit_message>
<xml_diff>
--- a/Data Input Pengujian/data.xlsx
+++ b/Data Input Pengujian/data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Python\odooCompressionTest\Data Input Pengujian\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{642CAFBF-97CF-4E33-A6B1-DD755D7AF778}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20762F44-3352-46ED-A5BC-7AF78D299752}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="55">
   <si>
     <t>Tanggal</t>
   </si>
@@ -52,31 +52,142 @@
     <t>Kode Benda Uji</t>
   </si>
   <si>
-    <t>13-01-2026</t>
-  </si>
-  <si>
-    <t>TATA / K 400 / AD PTB</t>
-  </si>
-  <si>
-    <t>VINFAST INTERNAL ROAD PACKAGE 1</t>
+    <t xml:space="preserve"> Slump 12.0 +2.0/-2.0</t>
+  </si>
+  <si>
+    <t>TM 944</t>
+  </si>
+  <si>
+    <t>Patimban Port Development Project Package 6 : Container Terminal No.2 Construction</t>
+  </si>
+  <si>
+    <t>Class A-2 NFA</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Slump 5.0 +5.0/-0.0</t>
+  </si>
+  <si>
+    <t>JALAN TOL AKSES PATIMBAN PAKET 4</t>
+  </si>
+  <si>
+    <t>TM 852</t>
+  </si>
+  <si>
+    <t>Class B-2 NFA</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Slump 55.0 +10.0/-0.0</t>
+  </si>
+  <si>
+    <t>AGUS</t>
+  </si>
+  <si>
+    <t>2026-06-02</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/06-2026/04655</t>
+  </si>
+  <si>
+    <t>HK - JAKON JO / PILEHEAD R11 - R15 OP 6 STA 32+048 / CLASS B-1 / AD PTB</t>
+  </si>
+  <si>
+    <t>Pembangunan Jalan Tol Akses Patimban Paket 3</t>
   </si>
   <si>
     <t>TAUFIQ</t>
   </si>
   <si>
-    <t>K-400 FA</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Slump 12.0 +1.5/-1.5</t>
-  </si>
-  <si>
-    <t>DOCKET/PTB/01-2026/00445</t>
-  </si>
-  <si>
-    <t>TM 601</t>
-  </si>
-  <si>
-    <t>13-01-2026 16:44:35</t>
+    <t>Class B-1 FA</t>
+  </si>
+  <si>
+    <t>TM 590</t>
+  </si>
+  <si>
+    <t>2026-06-02 19:19:08</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/06-2026/04658</t>
+  </si>
+  <si>
+    <t>2026-06-02 20:02:32</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/06-2026/04665</t>
+  </si>
+  <si>
+    <t>TM 902</t>
+  </si>
+  <si>
+    <t>2026-06-02 21:30:19</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/06-2026/04628</t>
+  </si>
+  <si>
+    <t>PTRPWJ / RIGID PAV - 14164 / CLASS A-2 / AD PTB</t>
+  </si>
+  <si>
+    <t>2026-06-02 14:42:48</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/06-2026/04632</t>
+  </si>
+  <si>
+    <t>TM 894</t>
+  </si>
+  <si>
+    <t>2026-06-02 15:28:20</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/06-2026/04638</t>
+  </si>
+  <si>
+    <t>2026-06-02 16:28:33</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/06-2026/04648</t>
+  </si>
+  <si>
+    <t>2026-06-02 18:08:44</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/06-2026/04661</t>
+  </si>
+  <si>
+    <t>2026-06-02 20:46:50</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/06-2026/04669</t>
+  </si>
+  <si>
+    <t>2026-06-02 21:59:53</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/06-2026/04641</t>
+  </si>
+  <si>
+    <t>WIKA - ADHI JO / BP P1 1A MB21 / CLASS B-2 SCC / AD PTB</t>
+  </si>
+  <si>
+    <t>NANDA</t>
+  </si>
+  <si>
+    <t>2026-06-02 17:02:51</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/06-2026/04644</t>
+  </si>
+  <si>
+    <t>2026-06-02 17:34:26</t>
+  </si>
+  <si>
+    <t>DOCKET/PTB/06-2026/04649</t>
+  </si>
+  <si>
+    <t>TM 813</t>
+  </si>
+  <si>
+    <t>2026-06-02 18:17:02</t>
   </si>
 </sst>
 </file>
@@ -450,7 +561,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.7109375" customWidth="1"/>
@@ -492,35 +603,358 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G2" t="s">
         <v>9</v>
       </c>
-      <c r="B2" t="s">
+      <c r="H2" t="s">
+        <v>25</v>
+      </c>
+      <c r="I2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" t="s">
+        <v>23</v>
+      </c>
+      <c r="F3" t="s">
+        <v>24</v>
+      </c>
+      <c r="G3" t="s">
+        <v>9</v>
+      </c>
+      <c r="H3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" t="s">
+        <v>24</v>
+      </c>
+      <c r="G4" t="s">
+        <v>9</v>
+      </c>
+      <c r="H4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G5" t="s">
+        <v>13</v>
+      </c>
+      <c r="H5" t="s">
         <v>15</v>
       </c>
-      <c r="C2" t="s">
+      <c r="I5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" t="s">
+        <v>13</v>
+      </c>
+      <c r="H6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C7" t="s">
+        <v>33</v>
+      </c>
+      <c r="D7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" t="s">
+        <v>18</v>
+      </c>
+      <c r="F7" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" t="s">
+        <v>13</v>
+      </c>
+      <c r="H7" t="s">
+        <v>15</v>
+      </c>
+      <c r="I7" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H8" t="s">
         <v>10</v>
       </c>
-      <c r="D2" t="s">
+      <c r="I8" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" t="s">
+        <v>33</v>
+      </c>
+      <c r="D9" t="s">
         <v>11</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E9" t="s">
+        <v>18</v>
+      </c>
+      <c r="F9" t="s">
         <v>12</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G9" t="s">
         <v>13</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H9" t="s">
+        <v>15</v>
+      </c>
+      <c r="I9" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10" t="s">
+        <v>33</v>
+      </c>
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" t="s">
+        <v>18</v>
+      </c>
+      <c r="F10" t="s">
+        <v>12</v>
+      </c>
+      <c r="G10" t="s">
+        <v>13</v>
+      </c>
+      <c r="H10" t="s">
+        <v>10</v>
+      </c>
+      <c r="I10" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" t="s">
+        <v>46</v>
+      </c>
+      <c r="C11" t="s">
+        <v>47</v>
+      </c>
+      <c r="D11" t="s">
         <v>14</v>
       </c>
-      <c r="H2" t="s">
+      <c r="E11" t="s">
+        <v>48</v>
+      </c>
+      <c r="F11" t="s">
         <v>16</v>
       </c>
-      <c r="I2" t="s">
+      <c r="G11" t="s">
         <v>17</v>
       </c>
+      <c r="H11" t="s">
+        <v>36</v>
+      </c>
+      <c r="I11" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" t="s">
+        <v>50</v>
+      </c>
+      <c r="C12" t="s">
+        <v>47</v>
+      </c>
+      <c r="D12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E12" t="s">
+        <v>48</v>
+      </c>
+      <c r="F12" t="s">
+        <v>16</v>
+      </c>
+      <c r="G12" t="s">
+        <v>17</v>
+      </c>
+      <c r="H12" t="s">
+        <v>15</v>
+      </c>
+      <c r="I12" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" t="s">
+        <v>52</v>
+      </c>
+      <c r="C13" t="s">
+        <v>47</v>
+      </c>
+      <c r="D13" t="s">
+        <v>14</v>
+      </c>
+      <c r="E13" t="s">
+        <v>48</v>
+      </c>
+      <c r="F13" t="s">
+        <v>16</v>
+      </c>
+      <c r="G13" t="s">
+        <v>17</v>
+      </c>
+      <c r="H13" t="s">
+        <v>53</v>
+      </c>
+      <c r="I13" t="s">
+        <v>54</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:I1" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I34">
+      <sortCondition ref="C1"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>